<commit_message>
01 septiembre 2020 v1
</commit_message>
<xml_diff>
--- a/_downloads/c1e77bd95e5dc71eeae06195b59dc204/Ejemplos swap IRS y swap CCS.xlsx
+++ b/_downloads/c1e77bd95e5dc71eeae06195b59dc204/Ejemplos swap IRS y swap CCS.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23001"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="23029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\ITM\DERIVADOS FINANCIEROS\CLASES\Swap\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\migue\Dropbox\UNAL\DERIVADOS FINANCIEROS\CLASES\Swap\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{855F8728-5F88-479A-9EC7-569DFAD89FE4}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{42E18EA5-AA8B-43F8-9C43-B1B37288F826}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Ejemplo No. 1 Swap IRS" sheetId="1" r:id="rId1"/>
@@ -2102,8 +2102,8 @@
       <xdr:row>18</xdr:row>
       <xdr:rowOff>1250</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 53">
@@ -2528,7 +2528,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="5" name="CuadroTexto 53">
@@ -6669,8 +6669,8 @@
       <xdr:row>19</xdr:row>
       <xdr:rowOff>1251</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 53">
@@ -7095,7 +7095,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="9" name="CuadroTexto 53">
@@ -7254,8 +7254,8 @@
       <xdr:rowOff>152399</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="667555" cy="318036"/>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="10" name="CuadroTexto 9">
@@ -7397,7 +7397,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="10" name="CuadroTexto 9">
@@ -8612,7 +8612,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>5</xdr:col>
-      <xdr:colOff>783770</xdr:colOff>
+      <xdr:colOff>1094014</xdr:colOff>
       <xdr:row>28</xdr:row>
       <xdr:rowOff>228600</xdr:rowOff>
     </xdr:to>
@@ -8632,7 +8632,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="4000500" y="7255329"/>
-          <a:ext cx="1600199" cy="440871"/>
+          <a:ext cx="1910443" cy="440871"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8801,18 +8801,6 @@
             <a:t>= </a:t>
           </a:r>
           <a:r>
-            <a:rPr lang="es-CO" sz="1200" kern="1200">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>B</a:t>
-          </a:r>
-          <a:r>
             <a:rPr lang="es-CO" sz="1200" kern="1200" baseline="-25000">
               <a:solidFill>
                 <a:schemeClr val="dk1"/>
@@ -8822,19 +8810,7 @@
               <a:ea typeface="+mn-ea"/>
               <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>variable </a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-CO" sz="1200" kern="1200" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="dk1"/>
-              </a:solidFill>
-              <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
-            </a:rPr>
-            <a:t>- </a:t>
+            <a:t> </a:t>
           </a:r>
           <a:r>
             <a:rPr lang="es-CO" sz="1200">
@@ -8858,7 +8834,31 @@
               <a:ea typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
               <a:cs typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
             </a:rPr>
-            <a:t> </a:t>
+            <a:t> - </a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1800" kern="1200">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>B</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="es-CO" sz="1800" kern="1200" baseline="-25000">
+              <a:solidFill>
+                <a:schemeClr val="dk1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>variable</a:t>
           </a:r>
           <a:endParaRPr lang="es-CO" sz="1200" baseline="-25000">
             <a:latin typeface="Tahoma" panose="020B0604030504040204" pitchFamily="34" charset="0"/>
@@ -11258,8 +11258,8 @@
       <xdr:row>19</xdr:row>
       <xdr:rowOff>12137</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-      <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
+      <mc:Choice Requires="a14">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="11" name="CuadroTexto 53">
@@ -11684,7 +11684,7 @@
           </xdr:txBody>
         </xdr:sp>
       </mc:Choice>
-      <mc:Fallback>
+      <mc:Fallback xmlns="">
         <xdr:sp macro="" textlink="">
           <xdr:nvSpPr>
             <xdr:cNvPr id="11" name="CuadroTexto 53">

</xml_diff>